<commit_message>
Add Information Theory, Inference and Learning Algorithms (MacKay)
n=58, Not started, 642 pp (Amazon), relevance 3. Not on a photographed shelf
(shelf=null); viewer now renders null shelf as an em dash.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/exports/Book_Inventory.xlsx
+++ b/exports/Book_Inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Books" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Books'!$A$1:$H$58</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Books'!$A$1:$H$59</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -550,7 +550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H58"/>
+  <dimension ref="A1:H59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2543,8 +2543,40 @@
         </is>
       </c>
     </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>Information Theory, Inference and Learning Algorithms</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>David J. C. MacKay</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="n"/>
+      <c r="E59" s="3" t="inlineStr">
+        <is>
+          <t>Economics &amp; Quant Methods</t>
+        </is>
+      </c>
+      <c r="F59" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="G59" s="2" t="n">
+        <v>642</v>
+      </c>
+      <c r="H59" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H58"/>
+  <autoFilter ref="A1:H59"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Replace 1-5 relevance score with four research buckets
Immediately relevant (8) / Will be relevant (12) / Maybe relevant (10) / For fun (28).
Subject category retained as a separate column.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/exports/Book_Inventory.xlsx
+++ b/exports/Book_Inventory.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -40,7 +40,7 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00843C0C"/>
+      <color rgb="00595959"/>
       <sz val="10"/>
     </font>
     <font>
@@ -63,7 +63,7 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00595959"/>
+      <color rgb="0006611F"/>
       <sz val="10"/>
     </font>
     <font>
@@ -72,14 +72,8 @@
       <color rgb="00006100"/>
       <sz val="10"/>
     </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00375623"/>
-      <sz val="10"/>
-    </font>
   </fonts>
-  <fills count="10">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -93,7 +87,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FCE4D6"/>
+        <fgColor rgb="00ECECEC"/>
       </patternFill>
     </fill>
     <fill>
@@ -113,17 +107,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E7E6E6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00C6EFCE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D6E9C6"/>
       </patternFill>
     </fill>
   </fills>
@@ -165,24 +149,24 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -558,8 +542,8 @@
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="7" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
@@ -591,7 +575,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Relevance (1-5)</t>
+          <t>Research Relevance</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -627,8 +611,10 @@
           <t>History</t>
         </is>
       </c>
-      <c r="F2" s="4" t="n">
-        <v>2</v>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>For fun</t>
+        </is>
       </c>
       <c r="G2" s="2" t="n">
         <v>752</v>
@@ -661,8 +647,10 @@
           <t>Politics &amp; Philosophy</t>
         </is>
       </c>
-      <c r="F3" s="6" t="n">
-        <v>3</v>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>Maybe relevant</t>
+        </is>
       </c>
       <c r="G3" s="2" t="n">
         <v>560</v>
@@ -695,8 +683,10 @@
           <t>Science &amp; Tech</t>
         </is>
       </c>
-      <c r="F4" s="4" t="n">
-        <v>2</v>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>For fun</t>
+        </is>
       </c>
       <c r="G4" s="2" t="n">
         <v>432</v>
@@ -729,8 +719,10 @@
           <t>Economics &amp; Quant Methods</t>
         </is>
       </c>
-      <c r="F5" s="6" t="n">
-        <v>3</v>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>Maybe relevant</t>
+        </is>
       </c>
       <c r="G5" s="2" t="n">
         <v>384</v>
@@ -763,8 +755,10 @@
           <t>Politics &amp; Philosophy</t>
         </is>
       </c>
-      <c r="F6" s="6" t="n">
-        <v>3</v>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>Maybe relevant</t>
+        </is>
       </c>
       <c r="G6" s="2" t="n">
         <v>328</v>
@@ -797,8 +791,10 @@
           <t>Arts, Media &amp; Essays</t>
         </is>
       </c>
-      <c r="F7" s="8" t="n">
-        <v>1</v>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>For fun</t>
+        </is>
       </c>
       <c r="G7" s="2" t="n">
         <v>256</v>
@@ -831,8 +827,10 @@
           <t>Poverty &amp; Social Policy</t>
         </is>
       </c>
-      <c r="F8" s="9" t="n">
-        <v>5</v>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>Immediately relevant</t>
+        </is>
       </c>
       <c r="G8" s="2" t="n">
         <v>456</v>
@@ -865,8 +863,10 @@
           <t>Poverty &amp; Social Policy</t>
         </is>
       </c>
-      <c r="F9" s="10" t="n">
-        <v>4</v>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>Will be relevant</t>
+        </is>
       </c>
       <c r="G9" s="2" t="n">
         <v>448</v>
@@ -899,13 +899,15 @@
           <t>Child Welfare &amp; Foster Care</t>
         </is>
       </c>
-      <c r="F10" s="9" t="n">
-        <v>5</v>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>Immediately relevant</t>
+        </is>
       </c>
       <c r="G10" s="2" t="n">
         <v>296</v>
       </c>
-      <c r="H10" s="9" t="inlineStr">
+      <c r="H10" s="10" t="inlineStr">
         <is>
           <t>Finished</t>
         </is>
@@ -933,8 +935,10 @@
           <t>Poverty &amp; Social Policy</t>
         </is>
       </c>
-      <c r="F11" s="9" t="n">
-        <v>5</v>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>Immediately relevant</t>
+        </is>
       </c>
       <c r="G11" s="2" t="n">
         <v>368</v>
@@ -967,13 +971,15 @@
           <t>Poverty &amp; Social Policy</t>
         </is>
       </c>
-      <c r="F12" s="10" t="n">
-        <v>4</v>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>Will be relevant</t>
+        </is>
       </c>
       <c r="G12" s="2" t="n">
         <v>480</v>
       </c>
-      <c r="H12" s="9" t="inlineStr">
+      <c r="H12" s="10" t="inlineStr">
         <is>
           <t>Finished</t>
         </is>
@@ -1001,13 +1007,15 @@
           <t>Writing &amp; Craft</t>
         </is>
       </c>
-      <c r="F13" s="4" t="n">
-        <v>2</v>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>Maybe relevant</t>
+        </is>
       </c>
       <c r="G13" s="2" t="n">
         <v>208</v>
       </c>
-      <c r="H13" s="9" t="inlineStr">
+      <c r="H13" s="10" t="inlineStr">
         <is>
           <t>Finished</t>
         </is>
@@ -1035,8 +1043,10 @@
           <t>Public Finance &amp; Tax</t>
         </is>
       </c>
-      <c r="F14" s="10" t="n">
-        <v>4</v>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t>Will be relevant</t>
+        </is>
       </c>
       <c r="G14" s="2" t="n">
         <v>568</v>
@@ -1069,8 +1079,10 @@
           <t>Arts, Media &amp; Essays</t>
         </is>
       </c>
-      <c r="F15" s="8" t="n">
-        <v>1</v>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>For fun</t>
+        </is>
       </c>
       <c r="G15" s="2" t="n">
         <v>352</v>
@@ -1103,8 +1115,10 @@
           <t>Public Finance &amp; Tax</t>
         </is>
       </c>
-      <c r="F16" s="9" t="n">
-        <v>5</v>
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>Will be relevant</t>
+        </is>
       </c>
       <c r="G16" s="2" t="n">
         <v>536</v>
@@ -1137,8 +1151,10 @@
           <t>History</t>
         </is>
       </c>
-      <c r="F17" s="4" t="n">
-        <v>2</v>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>For fun</t>
+        </is>
       </c>
       <c r="G17" s="2" t="n">
         <v>464</v>
@@ -1171,8 +1187,10 @@
           <t>Fiction</t>
         </is>
       </c>
-      <c r="F18" s="8" t="n">
-        <v>1</v>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>For fun</t>
+        </is>
       </c>
       <c r="G18" s="2" t="n">
         <v>576</v>
@@ -1205,8 +1223,10 @@
           <t>Poverty &amp; Social Policy</t>
         </is>
       </c>
-      <c r="F19" s="9" t="n">
-        <v>5</v>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>Immediately relevant</t>
+        </is>
       </c>
       <c r="G19" s="2" t="n">
         <v>336</v>
@@ -1239,8 +1259,10 @@
           <t>History</t>
         </is>
       </c>
-      <c r="F20" s="4" t="n">
-        <v>2</v>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>For fun</t>
+        </is>
       </c>
       <c r="G20" s="2" t="n">
         <v>688</v>
@@ -1273,8 +1295,10 @@
           <t>History</t>
         </is>
       </c>
-      <c r="F21" s="8" t="n">
-        <v>1</v>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>For fun</t>
+        </is>
       </c>
       <c r="G21" s="2" t="n">
         <v>352</v>
@@ -1307,8 +1331,10 @@
           <t>Urban &amp; Housing</t>
         </is>
       </c>
-      <c r="F22" s="10" t="n">
-        <v>4</v>
+      <c r="F22" s="9" t="inlineStr">
+        <is>
+          <t>Will be relevant</t>
+        </is>
       </c>
       <c r="G22" s="2" t="n">
         <v>352</v>
@@ -1341,8 +1367,10 @@
           <t>Science &amp; Tech</t>
         </is>
       </c>
-      <c r="F23" s="4" t="n">
-        <v>2</v>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>For fun</t>
+        </is>
       </c>
       <c r="G23" s="2" t="n">
         <v>777</v>
@@ -1375,8 +1403,10 @@
           <t>Arts, Media &amp; Essays</t>
         </is>
       </c>
-      <c r="F24" s="8" t="n">
-        <v>1</v>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>For fun</t>
+        </is>
       </c>
       <c r="G24" s="2" t="n">
         <v>480</v>
@@ -1409,8 +1439,10 @@
           <t>Fiction</t>
         </is>
       </c>
-      <c r="F25" s="8" t="n">
-        <v>1</v>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>For fun</t>
+        </is>
       </c>
       <c r="G25" s="2" t="n">
         <v>152</v>
@@ -1443,8 +1475,10 @@
           <t>Poverty &amp; Social Policy</t>
         </is>
       </c>
-      <c r="F26" s="10" t="n">
-        <v>4</v>
+      <c r="F26" s="9" t="inlineStr">
+        <is>
+          <t>Will be relevant</t>
+        </is>
       </c>
       <c r="G26" s="2" t="n">
         <v>232</v>
@@ -1477,8 +1511,10 @@
           <t>Fiction</t>
         </is>
       </c>
-      <c r="F27" s="8" t="n">
-        <v>1</v>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>For fun</t>
+        </is>
       </c>
       <c r="G27" s="2" t="n">
         <v>320</v>
@@ -1511,13 +1547,15 @@
           <t>Poverty &amp; Social Policy</t>
         </is>
       </c>
-      <c r="F28" s="6" t="n">
-        <v>3</v>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>Maybe relevant</t>
+        </is>
       </c>
       <c r="G28" s="2" t="n">
         <v>288</v>
       </c>
-      <c r="H28" s="9" t="inlineStr">
+      <c r="H28" s="10" t="inlineStr">
         <is>
           <t>Finished</t>
         </is>
@@ -1545,8 +1583,10 @@
           <t>Fiction</t>
         </is>
       </c>
-      <c r="F29" s="8" t="n">
-        <v>1</v>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>For fun</t>
+        </is>
       </c>
       <c r="G29" s="2" t="n">
         <v>320</v>
@@ -1579,8 +1619,10 @@
           <t>Fiction</t>
         </is>
       </c>
-      <c r="F30" s="8" t="n">
-        <v>1</v>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>For fun</t>
+        </is>
       </c>
       <c r="G30" s="2" t="n">
         <v>304</v>
@@ -1613,8 +1655,10 @@
           <t>Economics &amp; Quant Methods</t>
         </is>
       </c>
-      <c r="F31" s="9" t="n">
-        <v>5</v>
+      <c r="F31" s="9" t="inlineStr">
+        <is>
+          <t>Will be relevant</t>
+        </is>
       </c>
       <c r="G31" s="2" t="n">
         <v>320</v>
@@ -1647,8 +1691,10 @@
           <t>Writing &amp; Craft</t>
         </is>
       </c>
-      <c r="F32" s="4" t="n">
-        <v>2</v>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>For fun</t>
+        </is>
       </c>
       <c r="G32" s="2" t="n">
         <v>208</v>
@@ -1681,8 +1727,10 @@
           <t>History</t>
         </is>
       </c>
-      <c r="F33" s="4" t="n">
-        <v>2</v>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>For fun</t>
+        </is>
       </c>
       <c r="G33" s="2" t="n">
         <v>480</v>
@@ -1715,8 +1763,10 @@
           <t>Economics &amp; Quant Methods</t>
         </is>
       </c>
-      <c r="F34" s="6" t="n">
-        <v>3</v>
+      <c r="F34" s="6" t="inlineStr">
+        <is>
+          <t>Maybe relevant</t>
+        </is>
       </c>
       <c r="G34" s="2" t="n">
         <v>378</v>
@@ -1749,8 +1799,10 @@
           <t>Science &amp; Tech</t>
         </is>
       </c>
-      <c r="F35" s="8" t="n">
-        <v>1</v>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>For fun</t>
+        </is>
       </c>
       <c r="G35" s="2" t="n">
         <v>696</v>
@@ -1783,8 +1835,10 @@
           <t>Urban &amp; Housing</t>
         </is>
       </c>
-      <c r="F36" s="6" t="n">
-        <v>3</v>
+      <c r="F36" s="6" t="inlineStr">
+        <is>
+          <t>Maybe relevant</t>
+        </is>
       </c>
       <c r="G36" s="2" t="n">
         <v>512</v>
@@ -1817,8 +1871,10 @@
           <t>Science &amp; Tech</t>
         </is>
       </c>
-      <c r="F37" s="4" t="n">
-        <v>2</v>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>For fun</t>
+        </is>
       </c>
       <c r="G37" s="2" t="n">
         <v>592</v>
@@ -1851,8 +1907,10 @@
           <t>Poverty &amp; Social Policy</t>
         </is>
       </c>
-      <c r="F38" s="9" t="n">
-        <v>5</v>
+      <c r="F38" s="8" t="inlineStr">
+        <is>
+          <t>Immediately relevant</t>
+        </is>
       </c>
       <c r="G38" s="2" t="n">
         <v>296</v>
@@ -1885,13 +1943,15 @@
           <t>Science &amp; Tech</t>
         </is>
       </c>
-      <c r="F39" s="4" t="n">
-        <v>2</v>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>For fun</t>
+        </is>
       </c>
       <c r="G39" s="2" t="n">
         <v>480</v>
       </c>
-      <c r="H39" s="9" t="inlineStr">
+      <c r="H39" s="10" t="inlineStr">
         <is>
           <t>Finished</t>
         </is>
@@ -1919,8 +1979,10 @@
           <t>Economics &amp; Quant Methods</t>
         </is>
       </c>
-      <c r="F40" s="10" t="n">
-        <v>4</v>
+      <c r="F40" s="9" t="inlineStr">
+        <is>
+          <t>Will be relevant</t>
+        </is>
       </c>
       <c r="G40" s="2" t="n">
         <v>745</v>
@@ -1953,8 +2015,10 @@
           <t>Child Welfare &amp; Foster Care</t>
         </is>
       </c>
-      <c r="F41" s="9" t="n">
-        <v>5</v>
+      <c r="F41" s="8" t="inlineStr">
+        <is>
+          <t>Immediately relevant</t>
+        </is>
       </c>
       <c r="G41" s="2" t="n">
         <v>624</v>
@@ -1987,8 +2051,10 @@
           <t>Science &amp; Tech</t>
         </is>
       </c>
-      <c r="F42" s="4" t="n">
-        <v>2</v>
+      <c r="F42" s="4" t="inlineStr">
+        <is>
+          <t>For fun</t>
+        </is>
       </c>
       <c r="G42" s="2" t="n">
         <v>400</v>
@@ -2021,8 +2087,10 @@
           <t>Economics &amp; Quant Methods</t>
         </is>
       </c>
-      <c r="F43" s="10" t="n">
-        <v>4</v>
+      <c r="F43" s="9" t="inlineStr">
+        <is>
+          <t>Will be relevant</t>
+        </is>
       </c>
       <c r="G43" s="2" t="n">
         <v>288</v>
@@ -2055,13 +2123,15 @@
           <t>Urban &amp; Housing</t>
         </is>
       </c>
-      <c r="F44" s="6" t="n">
-        <v>3</v>
+      <c r="F44" s="4" t="inlineStr">
+        <is>
+          <t>For fun</t>
+        </is>
       </c>
       <c r="G44" s="2" t="n">
         <v>400</v>
       </c>
-      <c r="H44" s="9" t="inlineStr">
+      <c r="H44" s="10" t="inlineStr">
         <is>
           <t>Finished</t>
         </is>
@@ -2089,8 +2159,10 @@
           <t>History</t>
         </is>
       </c>
-      <c r="F45" s="4" t="n">
-        <v>2</v>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>For fun</t>
+        </is>
       </c>
       <c r="G45" s="2" t="n">
         <v>464</v>
@@ -2123,8 +2195,10 @@
           <t>Economics &amp; Quant Methods</t>
         </is>
       </c>
-      <c r="F46" s="9" t="n">
-        <v>5</v>
+      <c r="F46" s="9" t="inlineStr">
+        <is>
+          <t>Will be relevant</t>
+        </is>
       </c>
       <c r="G46" s="2" t="n">
         <v>224</v>
@@ -2157,8 +2231,10 @@
           <t>Politics &amp; Philosophy</t>
         </is>
       </c>
-      <c r="F47" s="4" t="n">
-        <v>2</v>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>For fun</t>
+        </is>
       </c>
       <c r="G47" s="2" t="n">
         <v>256</v>
@@ -2191,8 +2267,10 @@
           <t>Politics &amp; Philosophy</t>
         </is>
       </c>
-      <c r="F48" s="4" t="n">
-        <v>2</v>
+      <c r="F48" s="4" t="inlineStr">
+        <is>
+          <t>For fun</t>
+        </is>
       </c>
       <c r="G48" s="2" t="n">
         <v>496</v>
@@ -2225,8 +2303,10 @@
           <t>History</t>
         </is>
       </c>
-      <c r="F49" s="6" t="n">
-        <v>3</v>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>For fun</t>
+        </is>
       </c>
       <c r="G49" s="2" t="n">
         <v>480</v>
@@ -2259,8 +2339,10 @@
           <t>Politics &amp; Philosophy</t>
         </is>
       </c>
-      <c r="F50" s="6" t="n">
-        <v>3</v>
+      <c r="F50" s="6" t="inlineStr">
+        <is>
+          <t>Maybe relevant</t>
+        </is>
       </c>
       <c r="G50" s="2" t="n">
         <v>160</v>
@@ -2293,8 +2375,10 @@
           <t>Politics &amp; Philosophy</t>
         </is>
       </c>
-      <c r="F51" s="4" t="n">
-        <v>2</v>
+      <c r="F51" s="4" t="inlineStr">
+        <is>
+          <t>For fun</t>
+        </is>
       </c>
       <c r="G51" s="2" t="n">
         <v>424</v>
@@ -2327,8 +2411,10 @@
           <t>Urban &amp; Housing</t>
         </is>
       </c>
-      <c r="F52" s="10" t="n">
-        <v>4</v>
+      <c r="F52" s="9" t="inlineStr">
+        <is>
+          <t>Will be relevant</t>
+        </is>
       </c>
       <c r="G52" s="2" t="n">
         <v>335</v>
@@ -2361,8 +2447,10 @@
           <t>History</t>
         </is>
       </c>
-      <c r="F53" s="8" t="n">
-        <v>1</v>
+      <c r="F53" s="4" t="inlineStr">
+        <is>
+          <t>For fun</t>
+        </is>
       </c>
       <c r="G53" s="2" t="n">
         <v>336</v>
@@ -2395,13 +2483,15 @@
           <t>Urban &amp; Housing</t>
         </is>
       </c>
-      <c r="F54" s="9" t="n">
-        <v>5</v>
+      <c r="F54" s="8" t="inlineStr">
+        <is>
+          <t>Immediately relevant</t>
+        </is>
       </c>
       <c r="G54" s="2" t="n">
         <v>288</v>
       </c>
-      <c r="H54" s="9" t="inlineStr">
+      <c r="H54" s="10" t="inlineStr">
         <is>
           <t>Finished</t>
         </is>
@@ -2429,8 +2519,10 @@
           <t>Urban &amp; Housing</t>
         </is>
       </c>
-      <c r="F55" s="6" t="n">
-        <v>3</v>
+      <c r="F55" s="6" t="inlineStr">
+        <is>
+          <t>Maybe relevant</t>
+        </is>
       </c>
       <c r="G55" s="2" t="n">
         <v>552</v>
@@ -2463,8 +2555,10 @@
           <t>Child Welfare &amp; Foster Care</t>
         </is>
       </c>
-      <c r="F56" s="9" t="n">
-        <v>5</v>
+      <c r="F56" s="8" t="inlineStr">
+        <is>
+          <t>Immediately relevant</t>
+        </is>
       </c>
       <c r="G56" s="2" t="n">
         <v>496</v>
@@ -2497,8 +2591,10 @@
           <t>Urban &amp; Housing</t>
         </is>
       </c>
-      <c r="F57" s="10" t="n">
-        <v>4</v>
+      <c r="F57" s="9" t="inlineStr">
+        <is>
+          <t>Will be relevant</t>
+        </is>
       </c>
       <c r="G57" s="2" t="n">
         <v>400</v>
@@ -2531,13 +2627,15 @@
           <t>Fiction</t>
         </is>
       </c>
-      <c r="F58" s="4" t="n">
-        <v>2</v>
+      <c r="F58" s="4" t="inlineStr">
+        <is>
+          <t>For fun</t>
+        </is>
       </c>
       <c r="G58" s="2" t="n">
         <v>560</v>
       </c>
-      <c r="H58" s="9" t="inlineStr">
+      <c r="H58" s="10" t="inlineStr">
         <is>
           <t>Finished</t>
         </is>
@@ -2563,8 +2661,10 @@
           <t>Economics &amp; Quant Methods</t>
         </is>
       </c>
-      <c r="F59" s="6" t="n">
-        <v>3</v>
+      <c r="F59" s="6" t="inlineStr">
+        <is>
+          <t>Maybe relevant</t>
+        </is>
       </c>
       <c r="G59" s="2" t="n">
         <v>642</v>

</xml_diff>

<commit_message>
Add 4 books: Addiction by Design (started), Liberalism as a Way of Life, The Power to Destroy (Graetz), AI Snake Oil
n=59-62. Page counts verified on Amazon. Not on photographed shelves (shelf=null).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/exports/Book_Inventory.xlsx
+++ b/exports/Book_Inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Books" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Books'!$A$1:$H$59</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Books'!$A$1:$H$63</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H59"/>
+  <dimension ref="A1:H63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2675,8 +2675,144 @@
         </is>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>Addiction by Design</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>Natasha Dow Schüll</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="n"/>
+      <c r="E60" s="3" t="inlineStr">
+        <is>
+          <t>Science &amp; Tech</t>
+        </is>
+      </c>
+      <c r="F60" s="9" t="inlineStr">
+        <is>
+          <t>Will be relevant</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="n">
+        <v>472</v>
+      </c>
+      <c r="H60" s="5" t="inlineStr">
+        <is>
+          <t>Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>Liberalism as a Way of Life</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>Alexandre Lefebvre</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="n"/>
+      <c r="E61" s="3" t="inlineStr">
+        <is>
+          <t>Politics &amp; Philosophy</t>
+        </is>
+      </c>
+      <c r="F61" s="4" t="inlineStr">
+        <is>
+          <t>For fun</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="n">
+        <v>304</v>
+      </c>
+      <c r="H61" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>The Power to Destroy</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>Michael J. Graetz</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="n"/>
+      <c r="E62" s="3" t="inlineStr">
+        <is>
+          <t>Public Finance &amp; Tax</t>
+        </is>
+      </c>
+      <c r="F62" s="9" t="inlineStr">
+        <is>
+          <t>Will be relevant</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="n">
+        <v>368</v>
+      </c>
+      <c r="H62" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>AI Snake Oil</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>Arvind Narayanan &amp; Sayash Kapoor</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="n"/>
+      <c r="E63" s="3" t="inlineStr">
+        <is>
+          <t>Science &amp; Tech</t>
+        </is>
+      </c>
+      <c r="F63" s="6" t="inlineStr">
+        <is>
+          <t>Maybe relevant</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="n">
+        <v>360</v>
+      </c>
+      <c r="H63" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H59"/>
+  <autoFilter ref="A1:H63"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>